<commit_message>
sc: don't export autofilter in table if header is off
Creates invalid XLSX.

Regression from 143c39521567fd8078dfda2d2a14c90ccb431bdd.

Change-Id: I1f82fd4170bd44f33fb5a59aa78b012c25c5ff4c
Signed-off-by: Aron Budea <aron.budea@collabora.com>
Reviewed-on: https://gerrit.collaboraoffice.com/c/online/+/12556
Tested-by: Jenkins CPCI <releng@collaboraoffice.com>
Reviewed-by: Balázs Varga <balazs.varga@collabora.com>
</commit_message>
<xml_diff>
--- a/engine/sc/qa/unit/data/xlsx/tableFilterButtonsOff.xlsx
+++ b/engine/sc/qa/unit/data/xlsx/tableFilterButtonsOff.xlsx
@@ -1,19 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\balu\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19FB7C2F-688E-44C6-87D1-C375F37A2173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +45,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <i/>
@@ -137,7 +132,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="CustomTS" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="CustomTS" pivot="0" count="4">
       <tableStyleElement type="headerRow" dxfId="3"/>
       <tableStyleElement type="totalRow" dxfId="2"/>
       <tableStyleElement type="lastColumn" dxfId="1"/>
@@ -156,16 +151,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DDFCB35-D833-4F40-9840-D9D37B468FD5}" name="Table1" displayName="Table1" ref="H6:J10" totalsRowShown="0">
-  <autoFilter ref="H6:J10" xr:uid="{8DDFCB35-D833-4F40-9840-D9D37B468FD5}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="H6:J10" totalsRowShown="0">
+  <autoFilter ref="H6:J10">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{D3850DB1-3612-4B1A-BE17-182BCBF40B37}" name="Data1"/>
-    <tableColumn id="2" xr3:uid="{8F2F2A06-8D57-4C2A-A9FF-BF2B1B453590}" name="Data2"/>
-    <tableColumn id="3" xr3:uid="{FCBA401A-B5F3-44EB-970D-AB053843878C}" name="Data3"/>
+    <tableColumn id="1" name="Data1"/>
+    <tableColumn id="2" name="Data2"/>
+    <tableColumn id="3" name="Data3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table13" displayName="Table13" ref="H7:J10" headerRowCount="0" totalsRowShown="0">
+  <tableColumns count="3">
+    <tableColumn id="1" name="Data1"/>
+    <tableColumn id="2" name="Data2"/>
+    <tableColumn id="3" name="Data3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -433,7 +439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="H6:J10"/>
   <sheetFormatPr defaultRowHeight="25.8" x14ac:dyDescent="0.5"/>
   <cols>
@@ -497,8 +503,70 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="H7:J10"/>
+  <sheetFormatPr defaultRowHeight="25.8" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="2" max="2" width="20.9375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="7" spans="8:10" x14ac:dyDescent="0.5">
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="8:10" x14ac:dyDescent="0.5">
+      <c r="H8">
+        <v>3</v>
+      </c>
+      <c r="I8">
+        <v>5</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="8:10" x14ac:dyDescent="0.5">
+      <c r="H9">
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <v>2</v>
+      </c>
+      <c r="J9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="8:10" x14ac:dyDescent="0.5">
+      <c r="H10">
+        <v>5</v>
+      </c>
+      <c r="I10">
+        <v>5</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>